<commit_message>
Fix Module 1 supporting-file friction: merge cm-profil-dapur-rara.txt into cm-template-kompetitor.txt as one self-contained, pre-filled Dapur Rara example (business + 3 fictional competitors + ready prompt + expected-result reference + brand voice), so students without their own business don't have to invent competitor data to do the exercise. Students with their own business now edit the same file in place instead of using a separate blank template. Updated HTML copy (Yang Kamu Butuhkan, step-row, Latihan, Output), PPTX slides 4-5, and course outline xlsx to match. Fixed stale 'Modul 2 sampai 7'/'Modul 7 Capstone' references left over from before the two-course split.
</commit_message>
<xml_diff>
--- a/Content-Marketing/Course-Level/Content-Marketing-Course-Outline.xlsx
+++ b/Content-Marketing/Course-Level/Content-Marketing-Course-Outline.xlsx
@@ -535,12 +535,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>cm-template-kompetitor.txt (atau cm-profil-dapur-rara.txt sebagai contoh)</t>
+          <t>cm-template-kompetitor.txt (sudah terisi contoh Dapur Rara, edit untuk bisnis sendiri)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Isi template dengan data 3 kompetitor nyata, termasuk palet warna dan mood/gaya visual. Minta Claude buat SWOT + gap + 3 variasi kalimat positioning. Simpan 1 di Claude Projects untuk dipakai di Modul 2-5.</t>
+          <t>Pakai contoh Dapur Rara langsung, atau ganti dulu isinya dengan data bisnis + 3 kompetitor nyata (termasuk palet warna dan mood/gaya visual). Paste ke Claude, minta SWOT + gap + 3 variasi kalimat positioning. Simpan 1 di Claude Projects untuk dipakai di Modul 2-5.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
M02: use Project Knowledge for product catalog continuity (positioning M1 + katalog M2 both auto-carry to M3-5); ripple fix to M3; update PPTX + outline xlsx to match
</commit_message>
<xml_diff>
--- a/Content-Marketing/Course-Level/Content-Marketing-Course-Outline.xlsx
+++ b/Content-Marketing/Course-Level/Content-Marketing-Course-Outline.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Membuat deskripsi produk marketplace yang SEO-friendly dan menjual, pakai positioning dari Modul 1 sebagai acuan.</t>
+          <t>Membuat deskripsi produk marketplace yang SEO-friendly dan menjual. Data produk disimpan di Project Knowledge yang sama dengan positioning Modul 1, jadi otomatis dipakai lagi di Modul 3-5.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -580,7 +580,7 @@
           <t>- Struktur deskripsi produk yang menjual (hook, keyword, spesifikasi, benefit vs fitur, CTA)
 - Kesalahan umum (copy dari supplier, fokus fitur teknis, tanpa keyword, terlalu panjang tanpa struktur)
 - Contoh prompt buruk vs baik
-- Cara kerja 5 langkah: isi CSV -&gt; upload ke Claude -&gt; tambah positioning + instruksi format -&gt; review keyword -&gt; paste &amp; track ranking</t>
+- Cara kerja 5 langkah: isi CSV -&gt; upload ke Project Knowledge (bukan cuma chat) -&gt; generate langsung (positioning &amp; data produk otomatis dari Project) -&gt; review keyword -&gt; paste &amp; track ranking</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -590,12 +590,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Isi CSV minimal 5 produk. Upload ke Claude, generate semua deskripsi sekaligus. Paste 1 deskripsi terbaik ke listing, cek ranking setelah 7 hari.</t>
+          <t>Isi CSV minimal 5 produk. Upload ke Project Knowledge dari Project yang sama dengan Modul 1, generate semua deskripsi sekaligus tanpa ketik ulang positioning. Paste 1 deskripsi terbaik ke listing, cek ranking setelah 7 hari.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Claude.ai (chat + upload CSV), Tokopedia/Shopee (paste manual)</t>
+          <t>Claude.ai (chat), Claude Projects (Project Knowledge: cm-data-produk.csv), Tokopedia/Shopee (paste manual)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Membangun sistem kalender konten Instagram 30 hari dalam 1 sesi, pakai positioning + daftar produk sebagai bahan. Termasuk setup Canva Connector dan opsi Claude membuat grafis sederhana langsung.</t>
+          <t>Membangun sistem kalender konten Instagram 30 hari dalam 1 sesi — positioning dan katalog produk sudah otomatis tersedia dari Project yang sama (Modul 1-2). Termasuk setup Canva Connector dan opsi Claude membuat grafis sederhana langsung.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Claude.ai (chat), Canva Connector, Claude Projects (baca positioning + identitas visual dari Modul 1)</t>
+          <t>Claude.ai (chat), Canva Connector, Claude Projects (baca positioning dari Modul 1 + katalog produk dari Modul 2, keduanya otomatis)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add copy-paste prompt-box to Latihan sections in M02-M05 (M01 intentionally excluded - prompt already lives in cm-template-kompetitor.txt); update M02 PPTX + outline xlsx to match
</commit_message>
<xml_diff>
--- a/Content-Marketing/Course-Level/Content-Marketing-Course-Outline.xlsx
+++ b/Content-Marketing/Course-Level/Content-Marketing-Course-Outline.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Isi CSV minimal 5 produk. Upload ke Project Knowledge dari Project yang sama dengan Modul 1, generate semua deskripsi sekaligus tanpa ketik ulang positioning. Paste 1 deskripsi terbaik ke listing, cek ranking setelah 7 hari.</t>
+          <t>Isi CSV minimal 5 produk. Upload ke Project Knowledge dari Project yang sama dengan Modul 1, lalu jalankan prompt siap-pakai di halaman kursus (copy-paste, sudah termasuk instruksi format). Paste 1 deskripsi terbaik ke listing, cek ranking setelah 7 hari.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Generate kalender konten Instagram 30 hari (16 post/bulan) dari positioning + daftar produk. Setup Canva Connector, buat 2-3 desain. Isi ke cm-kalender-konten.csv, jadwalkan minggu pertama.</t>
+          <t>Jalankan prompt siap-pakai di halaman kursus untuk generate kalender Instagram 30 hari (16 post/bulan) dari positioning + daftar produk yang sudah ada di Project. Setup Canva Connector, buat 2-3 desain. Isi ke cm-kalender-konten.csv, jadwalkan minggu pertama.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Buat 3 variasi copy iklan untuk 1 promo/produk di platform pilihan. Minta Claude buatkan desain Canva sesuai brand. Jalankan A/B test 3 hari, track CTR dan ROAS.</t>
+          <t>Jalankan prompt siap-pakai di halaman kursus (ganti [nama produk/promo], [diskon], dll dengan datamu) untuk 1 promo/produk di platform pilihan. Minta Claude buatkan desain Canva sesuai brand. Jalankan A/B test 3 hari, track CTR dan ROAS.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Tambahkan brand voice CS ke Claude Project dari Modul 1. Buat 10 template WhatsApp untuk skenario umum + minimal 2 draft email via Gmail Connector.</t>
+          <t>Jalankan prompt siap-pakai di halaman kursus untuk tambahkan brand voice CS ke Claude Project dari Modul 1, generate 10 template WhatsApp + 2 draft email sekaligus via Gmail Connector.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">

</xml_diff>